<commit_message>
feat: merge 210 elemental talents, proc matrix, and balanced costs to main
</commit_message>
<xml_diff>
--- a/Talentos_Fallen_Hero.xlsx
+++ b/Talentos_Fallen_Hero.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documentos\Repositórios\Fallen-Hero\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B48784A3-97CE-4164-9429-01B3BAC90940}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1361DE09-7B43-40DE-AF0B-069D565ECFD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A1D81212-02A5-4C62-B568-84DC2B032758}"/>
+    <workbookView xWindow="3330" yWindow="3330" windowWidth="21600" windowHeight="11385" xr2:uid="{A1D81212-02A5-4C62-B568-84DC2B032758}"/>
   </bookViews>
   <sheets>
     <sheet name="Talentos" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1058" uniqueCount="658">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1269" uniqueCount="660">
   <si>
     <t>id</t>
   </si>
@@ -2016,13 +2016,19 @@
   </si>
   <si>
     <t>Ativar Furia Ardente consome 30% do HP atual, mas dobra o bonus de dano de fogo nos primeiros 3s.</t>
+  </si>
+  <si>
+    <t>Status ImplementaÃ§Ã£o</t>
+  </si>
+  <si>
+    <t>IMPLEMENTADO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2069,8 +2075,15 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF245715"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2086,6 +2099,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFCFAF9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDAEDD4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2117,7 +2136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2158,7 +2177,11 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2495,7 +2518,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43E915D8-A9A5-4DC7-8FA7-F04EE98E54F2}">
-  <dimension ref="A1:H211"/>
+  <dimension ref="A1:I211"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.7109375" customWidth="1"/>
@@ -2505,9 +2528,10 @@
     <col min="5" max="5" width="30.7109375" customWidth="1"/>
     <col min="6" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2532,8 +2556,11 @@
       <c r="H1" s="1" t="s">
         <v>656</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="1" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -2549,11 +2576,16 @@
       <c r="E2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="14">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>10</v>
       </c>
@@ -2569,11 +2601,16 @@
       <c r="E3" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="14">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>13</v>
       </c>
@@ -2589,11 +2626,16 @@
       <c r="E4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="14">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>16</v>
       </c>
@@ -2609,11 +2651,16 @@
       <c r="E5" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="14">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>19</v>
       </c>
@@ -2629,11 +2676,16 @@
       <c r="E6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F6">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="F6" s="14">
+        <v>9</v>
+      </c>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>22</v>
       </c>
@@ -2649,11 +2701,16 @@
       <c r="E7" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="14">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>25</v>
       </c>
@@ -2669,17 +2726,20 @@
       <c r="E8" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="14">
         <v>1</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="14">
         <v>2</v>
       </c>
-      <c r="H8">
+      <c r="H8" s="14">
         <v>4</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I8" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>29</v>
       </c>
@@ -2695,17 +2755,20 @@
       <c r="E9" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="14">
         <v>1</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="14">
         <v>4</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="14">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I9" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>32</v>
       </c>
@@ -2721,11 +2784,16 @@
       <c r="E10" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="14">
         <v>5</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
+      <c r="I10" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>35</v>
       </c>
@@ -2741,11 +2809,16 @@
       <c r="E11" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="14">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
+      <c r="I11" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>38</v>
       </c>
@@ -2761,17 +2834,20 @@
       <c r="E12" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="14">
         <v>1</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="14">
         <v>4</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="14">
         <v>8</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="I12" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>42</v>
       </c>
@@ -2787,11 +2863,16 @@
       <c r="E13" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="14">
         <v>10</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G13" s="14"/>
+      <c r="H13" s="14"/>
+      <c r="I13" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>45</v>
       </c>
@@ -2807,11 +2888,16 @@
       <c r="E14" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="14">
         <v>8</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G14" s="14"/>
+      <c r="H14" s="14"/>
+      <c r="I14" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>48</v>
       </c>
@@ -2827,11 +2913,16 @@
       <c r="E15" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="14">
         <v>4</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G15" s="14"/>
+      <c r="H15" s="14"/>
+      <c r="I15" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>51</v>
       </c>
@@ -2847,11 +2938,16 @@
       <c r="E16" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="14">
         <v>6</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G16" s="14"/>
+      <c r="H16" s="14"/>
+      <c r="I16" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>54</v>
       </c>
@@ -2867,11 +2963,16 @@
       <c r="E17" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="14">
         <v>3</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14"/>
+      <c r="H17" s="14"/>
+      <c r="I17" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>57</v>
       </c>
@@ -2887,11 +2988,16 @@
       <c r="E18" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="14">
         <v>4</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
+      <c r="I18" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>60</v>
       </c>
@@ -2907,11 +3013,16 @@
       <c r="E19" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="14">
         <v>3</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
+      <c r="I19" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>63</v>
       </c>
@@ -2927,11 +3038,16 @@
       <c r="E20" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="14">
         <v>8</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
+      <c r="I20" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>67</v>
       </c>
@@ -2947,11 +3063,16 @@
       <c r="E21" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="14">
         <v>8</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G21" s="14"/>
+      <c r="H21" s="14"/>
+      <c r="I21" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>70</v>
       </c>
@@ -2967,11 +3088,16 @@
       <c r="E22" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="14">
         <v>6</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G22" s="14"/>
+      <c r="H22" s="14"/>
+      <c r="I22" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
         <v>73</v>
       </c>
@@ -2987,11 +3113,16 @@
       <c r="E23" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F23">
+      <c r="F23" s="14">
         <v>10</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G23" s="14"/>
+      <c r="H23" s="14"/>
+      <c r="I23" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>76</v>
       </c>
@@ -3007,11 +3138,16 @@
       <c r="E24" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="14">
         <v>3</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G24" s="14"/>
+      <c r="H24" s="14"/>
+      <c r="I24" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>78</v>
       </c>
@@ -3027,11 +3163,16 @@
       <c r="E25" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F25">
+      <c r="F25" s="14">
         <v>6</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G25" s="14"/>
+      <c r="H25" s="14"/>
+      <c r="I25" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>81</v>
       </c>
@@ -3047,11 +3188,16 @@
       <c r="E26" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F26">
+      <c r="F26" s="14">
         <v>2</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G26" s="14"/>
+      <c r="H26" s="14"/>
+      <c r="I26" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
         <v>84</v>
       </c>
@@ -3067,11 +3213,16 @@
       <c r="E27" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F27">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F27" s="14">
+        <v>9</v>
+      </c>
+      <c r="G27" s="14"/>
+      <c r="H27" s="14"/>
+      <c r="I27" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>87</v>
       </c>
@@ -3087,11 +3238,16 @@
       <c r="E28" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F28">
+      <c r="F28" s="14">
         <v>3</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G28" s="14"/>
+      <c r="H28" s="14"/>
+      <c r="I28" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
         <v>91</v>
       </c>
@@ -3107,11 +3263,16 @@
       <c r="E29" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F29">
+      <c r="F29" s="14">
         <v>5</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G29" s="14"/>
+      <c r="H29" s="14"/>
+      <c r="I29" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>94</v>
       </c>
@@ -3127,11 +3288,16 @@
       <c r="E30" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F30">
+      <c r="F30" s="14">
         <v>6</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G30" s="14"/>
+      <c r="H30" s="14"/>
+      <c r="I30" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
         <v>97</v>
       </c>
@@ -3147,11 +3313,16 @@
       <c r="E31" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F31">
+      <c r="F31" s="14">
         <v>2</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G31" s="14"/>
+      <c r="H31" s="14"/>
+      <c r="I31" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>100</v>
       </c>
@@ -3167,11 +3338,16 @@
       <c r="E32" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F32">
+      <c r="F32" s="14">
         <v>4</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G32" s="14"/>
+      <c r="H32" s="14"/>
+      <c r="I32" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
         <v>103</v>
       </c>
@@ -3187,11 +3363,16 @@
       <c r="E33" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F33">
+      <c r="F33" s="14">
         <v>7</v>
       </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G33" s="14"/>
+      <c r="H33" s="14"/>
+      <c r="I33" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>106</v>
       </c>
@@ -3207,17 +3388,20 @@
       <c r="E34" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="F34">
+      <c r="F34" s="14">
         <v>1</v>
       </c>
-      <c r="G34">
+      <c r="G34" s="14">
         <v>5</v>
       </c>
-      <c r="H34">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H34" s="14">
+        <v>9</v>
+      </c>
+      <c r="I34" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
         <v>109</v>
       </c>
@@ -3233,11 +3417,16 @@
       <c r="E35" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F35">
+      <c r="F35" s="14">
         <v>8</v>
       </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G35" s="14"/>
+      <c r="H35" s="14"/>
+      <c r="I35" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>112</v>
       </c>
@@ -3253,11 +3442,16 @@
       <c r="E36" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F36">
+      <c r="F36" s="14">
         <v>5</v>
       </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G36" s="14"/>
+      <c r="H36" s="14"/>
+      <c r="I36" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
         <v>116</v>
       </c>
@@ -3273,11 +3467,16 @@
       <c r="E37" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F37">
+      <c r="F37" s="14">
         <v>2</v>
       </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G37" s="14"/>
+      <c r="H37" s="14"/>
+      <c r="I37" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>119</v>
       </c>
@@ -3293,17 +3492,20 @@
       <c r="E38" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="F38">
+      <c r="F38" s="14">
         <v>3</v>
       </c>
-      <c r="G38">
+      <c r="G38" s="14">
         <v>8</v>
       </c>
-      <c r="H38">
+      <c r="H38" s="14">
         <v>12</v>
       </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I38" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
         <v>122</v>
       </c>
@@ -3319,11 +3521,16 @@
       <c r="E39" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F39">
+      <c r="F39" s="14">
         <v>6</v>
       </c>
-    </row>
-    <row r="40" spans="1:8" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G39" s="14"/>
+      <c r="H39" s="14"/>
+      <c r="I39" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>125</v>
       </c>
@@ -3339,11 +3546,16 @@
       <c r="E40" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F40">
+      <c r="F40" s="14">
         <v>2</v>
       </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G40" s="14"/>
+      <c r="H40" s="14"/>
+      <c r="I40" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
         <v>128</v>
       </c>
@@ -3359,11 +3571,16 @@
       <c r="E41" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F41">
+      <c r="F41" s="14">
         <v>6</v>
       </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G41" s="14"/>
+      <c r="H41" s="14"/>
+      <c r="I41" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>131</v>
       </c>
@@ -3379,17 +3596,20 @@
       <c r="E42" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F42">
+      <c r="F42" s="14">
         <v>1</v>
       </c>
-      <c r="G42">
+      <c r="G42" s="14">
         <v>2</v>
       </c>
-      <c r="H42">
+      <c r="H42" s="14">
         <v>4</v>
       </c>
-    </row>
-    <row r="43" spans="1:8" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="I42" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
         <v>134</v>
       </c>
@@ -3405,11 +3625,16 @@
       <c r="E43" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F43">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F43" s="14">
+        <v>9</v>
+      </c>
+      <c r="G43" s="14"/>
+      <c r="H43" s="14"/>
+      <c r="I43" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>137</v>
       </c>
@@ -3425,11 +3650,16 @@
       <c r="E44" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F44">
+      <c r="F44" s="14">
         <v>15</v>
       </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G44" s="14"/>
+      <c r="H44" s="14"/>
+      <c r="I44" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
         <v>140</v>
       </c>
@@ -3445,11 +3675,16 @@
       <c r="E45" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F45">
+      <c r="F45" s="14">
         <v>12</v>
       </c>
-    </row>
-    <row r="46" spans="1:8" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G45" s="14"/>
+      <c r="H45" s="14"/>
+      <c r="I45" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>143</v>
       </c>
@@ -3465,11 +3700,16 @@
       <c r="E46" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F46">
+      <c r="F46" s="14">
         <v>10</v>
       </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G46" s="14"/>
+      <c r="H46" s="14"/>
+      <c r="I46" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
         <v>146</v>
       </c>
@@ -3485,11 +3725,16 @@
       <c r="E47" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F47">
+      <c r="F47" s="14">
         <v>14</v>
       </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G47" s="14"/>
+      <c r="H47" s="14"/>
+      <c r="I47" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>149</v>
       </c>
@@ -3505,11 +3750,16 @@
       <c r="E48" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F48">
+      <c r="F48" s="14">
         <v>12</v>
       </c>
-    </row>
-    <row r="49" spans="1:8" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G48" s="14"/>
+      <c r="H48" s="14"/>
+      <c r="I48" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
         <v>152</v>
       </c>
@@ -3525,11 +3775,16 @@
       <c r="E49" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F49">
+      <c r="F49" s="14">
         <v>15</v>
       </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G49" s="14"/>
+      <c r="H49" s="14"/>
+      <c r="I49" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>155</v>
       </c>
@@ -3545,11 +3800,16 @@
       <c r="E50" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F50">
+      <c r="F50" s="14">
         <v>10</v>
       </c>
-    </row>
-    <row r="51" spans="1:8" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G50" s="14"/>
+      <c r="H50" s="14"/>
+      <c r="I50" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
         <v>158</v>
       </c>
@@ -3565,11 +3825,16 @@
       <c r="E51" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F51">
+      <c r="F51" s="14">
         <v>13</v>
       </c>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G51" s="14"/>
+      <c r="H51" s="14"/>
+      <c r="I51" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>161</v>
       </c>
@@ -3585,11 +3850,16 @@
       <c r="E52" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F52">
+      <c r="F52" s="14">
         <v>3</v>
       </c>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G52" s="14"/>
+      <c r="H52" s="14"/>
+      <c r="I52" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
         <v>165</v>
       </c>
@@ -3605,11 +3875,16 @@
       <c r="E53" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F53">
+      <c r="F53" s="14">
         <v>4</v>
       </c>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G53" s="14"/>
+      <c r="H53" s="14"/>
+      <c r="I53" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>168</v>
       </c>
@@ -3625,11 +3900,16 @@
       <c r="E54" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F54">
+      <c r="F54" s="14">
         <v>6</v>
       </c>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G54" s="14"/>
+      <c r="H54" s="14"/>
+      <c r="I54" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
         <v>171</v>
       </c>
@@ -3645,11 +3925,16 @@
       <c r="E55" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F55">
+      <c r="F55" s="14">
         <v>2</v>
       </c>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G55" s="14"/>
+      <c r="H55" s="14"/>
+      <c r="I55" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>174</v>
       </c>
@@ -3665,11 +3950,16 @@
       <c r="E56" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F56">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F56" s="14">
+        <v>9</v>
+      </c>
+      <c r="G56" s="14"/>
+      <c r="H56" s="14"/>
+      <c r="I56" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
         <v>177</v>
       </c>
@@ -3685,11 +3975,16 @@
       <c r="E57" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F57">
+      <c r="F57" s="14">
         <v>7</v>
       </c>
-    </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G57" s="14"/>
+      <c r="H57" s="14"/>
+      <c r="I57" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>180</v>
       </c>
@@ -3705,11 +4000,16 @@
       <c r="E58" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F58">
+      <c r="F58" s="14">
         <v>5</v>
       </c>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G58" s="14"/>
+      <c r="H58" s="14"/>
+      <c r="I58" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
         <v>183</v>
       </c>
@@ -3725,11 +4025,16 @@
       <c r="E59" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F59">
+      <c r="F59" s="14">
         <v>3</v>
       </c>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G59" s="14"/>
+      <c r="H59" s="14"/>
+      <c r="I59" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>186</v>
       </c>
@@ -3745,11 +4050,16 @@
       <c r="E60" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F60">
+      <c r="F60" s="14">
         <v>8</v>
       </c>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G60" s="14"/>
+      <c r="H60" s="14"/>
+      <c r="I60" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
         <v>189</v>
       </c>
@@ -3765,17 +4075,20 @@
       <c r="E61" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="F61">
+      <c r="F61" s="14">
         <v>1</v>
       </c>
-      <c r="G61">
+      <c r="G61" s="14">
         <v>3</v>
       </c>
-      <c r="H61">
+      <c r="H61" s="14">
         <v>7</v>
       </c>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I61" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>192</v>
       </c>
@@ -3791,11 +4104,16 @@
       <c r="E62" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F62">
+      <c r="F62" s="14">
         <v>4</v>
       </c>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G62" s="14"/>
+      <c r="H62" s="14"/>
+      <c r="I62" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
         <v>196</v>
       </c>
@@ -3811,11 +4129,16 @@
       <c r="E63" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F63">
+      <c r="F63" s="14">
         <v>5</v>
       </c>
-    </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G63" s="14"/>
+      <c r="H63" s="14"/>
+      <c r="I63" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>199</v>
       </c>
@@ -3831,11 +4154,16 @@
       <c r="E64" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F64">
+      <c r="F64" s="14">
         <v>3</v>
       </c>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G64" s="14"/>
+      <c r="H64" s="14"/>
+      <c r="I64" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
         <v>202</v>
       </c>
@@ -3851,11 +4179,16 @@
       <c r="E65" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F65">
+      <c r="F65" s="14">
         <v>6</v>
       </c>
-    </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G65" s="14"/>
+      <c r="H65" s="14"/>
+      <c r="I65" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>205</v>
       </c>
@@ -3871,11 +4204,16 @@
       <c r="E66" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F66">
+      <c r="F66" s="14">
         <v>4</v>
       </c>
-    </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G66" s="14"/>
+      <c r="H66" s="14"/>
+      <c r="I66" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
         <v>208</v>
       </c>
@@ -3891,11 +4229,16 @@
       <c r="E67" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F67">
+      <c r="F67" s="14">
         <v>7</v>
       </c>
-    </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G67" s="14"/>
+      <c r="H67" s="14"/>
+      <c r="I67" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>211</v>
       </c>
@@ -3911,11 +4254,16 @@
       <c r="E68" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F68">
+      <c r="F68" s="14">
         <v>5</v>
       </c>
-    </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G68" s="14"/>
+      <c r="H68" s="14"/>
+      <c r="I68" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
         <v>214</v>
       </c>
@@ -3931,11 +4279,16 @@
       <c r="E69" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F69">
+      <c r="F69" s="14">
         <v>8</v>
       </c>
-    </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G69" s="14"/>
+      <c r="H69" s="14"/>
+      <c r="I69" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>217</v>
       </c>
@@ -3951,11 +4304,16 @@
       <c r="E70" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F70">
+      <c r="F70" s="14">
         <v>4</v>
       </c>
-    </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G70" s="14"/>
+      <c r="H70" s="14"/>
+      <c r="I70" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
         <v>221</v>
       </c>
@@ -3971,11 +4329,16 @@
       <c r="E71" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F71">
+      <c r="F71" s="14">
         <v>6</v>
       </c>
-    </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G71" s="14"/>
+      <c r="H71" s="14"/>
+      <c r="I71" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>224</v>
       </c>
@@ -3991,11 +4354,16 @@
       <c r="E72" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F72">
+      <c r="F72" s="14">
         <v>4</v>
       </c>
-    </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G72" s="14"/>
+      <c r="H72" s="14"/>
+      <c r="I72" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
         <v>227</v>
       </c>
@@ -4011,11 +4379,16 @@
       <c r="E73" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F73">
+      <c r="F73" s="14">
         <v>3</v>
       </c>
-    </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G73" s="14"/>
+      <c r="H73" s="14"/>
+      <c r="I73" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>230</v>
       </c>
@@ -4031,11 +4404,16 @@
       <c r="E74" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F74">
+      <c r="F74" s="14">
         <v>8</v>
       </c>
-    </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G74" s="14"/>
+      <c r="H74" s="14"/>
+      <c r="I74" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
         <v>233</v>
       </c>
@@ -4051,11 +4429,16 @@
       <c r="E75" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F75">
+      <c r="F75" s="14">
         <v>4</v>
       </c>
-    </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G75" s="14"/>
+      <c r="H75" s="14"/>
+      <c r="I75" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>236</v>
       </c>
@@ -4071,11 +4454,16 @@
       <c r="E76" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F76">
+      <c r="F76" s="14">
         <v>7</v>
       </c>
-    </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G76" s="14"/>
+      <c r="H76" s="14"/>
+      <c r="I76" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
         <v>239</v>
       </c>
@@ -4091,11 +4479,16 @@
       <c r="E77" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F77">
+      <c r="F77" s="14">
         <v>12</v>
       </c>
-    </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G77" s="14"/>
+      <c r="H77" s="14"/>
+      <c r="I77" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>242</v>
       </c>
@@ -4111,11 +4504,16 @@
       <c r="E78" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F78">
+      <c r="F78" s="14">
         <v>4</v>
       </c>
-    </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G78" s="14"/>
+      <c r="H78" s="14"/>
+      <c r="I78" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
         <v>246</v>
       </c>
@@ -4131,17 +4529,20 @@
       <c r="E79" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="F79">
+      <c r="F79" s="14">
         <v>1</v>
       </c>
-      <c r="G79">
+      <c r="G79" s="14">
         <v>2</v>
       </c>
-      <c r="H79">
+      <c r="H79" s="14">
         <v>4</v>
       </c>
-    </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I79" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>249</v>
       </c>
@@ -4157,11 +4558,16 @@
       <c r="E80" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F80">
+      <c r="F80" s="14">
         <v>4</v>
       </c>
-    </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G80" s="14"/>
+      <c r="H80" s="14"/>
+      <c r="I80" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
         <v>252</v>
       </c>
@@ -4177,13 +4583,16 @@
       <c r="E81" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F81" s="14">
+      <c r="F81" s="16">
         <v>5</v>
       </c>
-      <c r="G81" s="14"/>
-      <c r="H81" s="14"/>
-    </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G81" s="16"/>
+      <c r="H81" s="16"/>
+      <c r="I81" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>255</v>
       </c>
@@ -4199,13 +4608,16 @@
       <c r="E82" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F82" s="14">
+      <c r="F82" s="16">
         <v>6</v>
       </c>
-      <c r="G82" s="14"/>
-      <c r="H82" s="14"/>
-    </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G82" s="16"/>
+      <c r="H82" s="16"/>
+      <c r="I82" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" s="7" t="s">
         <v>258</v>
       </c>
@@ -4221,13 +4633,16 @@
       <c r="E83" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F83" s="14">
+      <c r="F83" s="16">
         <v>6</v>
       </c>
-      <c r="G83" s="14"/>
-      <c r="H83" s="14"/>
-    </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G83" s="16"/>
+      <c r="H83" s="16"/>
+      <c r="I83" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>261</v>
       </c>
@@ -4243,13 +4658,16 @@
       <c r="E84" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F84" s="14">
+      <c r="F84" s="16">
         <v>8</v>
       </c>
-      <c r="G84" s="14"/>
-      <c r="H84" s="14"/>
-    </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G84" s="16"/>
+      <c r="H84" s="16"/>
+      <c r="I84" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" s="7" t="s">
         <v>264</v>
       </c>
@@ -4265,17 +4683,20 @@
       <c r="E85" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="F85" s="14">
+      <c r="F85" s="16">
         <v>1</v>
       </c>
-      <c r="G85" s="14">
+      <c r="G85" s="16">
         <v>3</v>
       </c>
-      <c r="H85" s="14">
+      <c r="H85" s="16">
         <v>7</v>
       </c>
-    </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I85" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>267</v>
       </c>
@@ -4291,13 +4712,16 @@
       <c r="E86" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F86" s="14">
+      <c r="F86" s="16">
         <v>4</v>
       </c>
-      <c r="G86" s="14"/>
-      <c r="H86" s="14"/>
-    </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G86" s="16"/>
+      <c r="H86" s="16"/>
+      <c r="I86" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" s="7" t="s">
         <v>271</v>
       </c>
@@ -4313,17 +4737,20 @@
       <c r="E87" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="F87" s="14">
+      <c r="F87" s="16">
         <v>2</v>
       </c>
-      <c r="G87" s="14">
+      <c r="G87" s="16">
         <v>5</v>
       </c>
-      <c r="H87" s="14">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H87" s="16">
+        <v>9</v>
+      </c>
+      <c r="I87" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>274</v>
       </c>
@@ -4339,13 +4766,16 @@
       <c r="E88" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F88" s="14">
+      <c r="F88" s="16">
         <v>6</v>
       </c>
-      <c r="G88" s="14"/>
-      <c r="H88" s="14"/>
-    </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G88" s="16"/>
+      <c r="H88" s="16"/>
+      <c r="I88" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" s="7" t="s">
         <v>277</v>
       </c>
@@ -4361,13 +4791,16 @@
       <c r="E89" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F89" s="14">
+      <c r="F89" s="16">
         <v>8</v>
       </c>
-      <c r="G89" s="14"/>
-      <c r="H89" s="14"/>
-    </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G89" s="16"/>
+      <c r="H89" s="16"/>
+      <c r="I89" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>280</v>
       </c>
@@ -4383,13 +4816,16 @@
       <c r="E90" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F90" s="14">
+      <c r="F90" s="16">
         <v>5</v>
       </c>
-      <c r="G90" s="14"/>
-      <c r="H90" s="14"/>
-    </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G90" s="16"/>
+      <c r="H90" s="16"/>
+      <c r="I90" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" s="7" t="s">
         <v>283</v>
       </c>
@@ -4405,13 +4841,16 @@
       <c r="E91" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F91" s="14">
+      <c r="F91" s="16">
         <v>3</v>
       </c>
-      <c r="G91" s="14"/>
-      <c r="H91" s="14"/>
-    </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G91" s="16"/>
+      <c r="H91" s="16"/>
+      <c r="I91" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
         <v>286</v>
       </c>
@@ -4427,13 +4866,16 @@
       <c r="E92" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F92" s="14">
+      <c r="F92" s="16">
         <v>7</v>
       </c>
-      <c r="G92" s="14"/>
-      <c r="H92" s="14"/>
-    </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G92" s="16"/>
+      <c r="H92" s="16"/>
+      <c r="I92" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" s="7" t="s">
         <v>289</v>
       </c>
@@ -4449,13 +4891,16 @@
       <c r="E93" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F93" s="14">
+      <c r="F93" s="16">
         <v>5</v>
       </c>
-      <c r="G93" s="14"/>
-      <c r="H93" s="14"/>
-    </row>
-    <row r="94" spans="1:8" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G93" s="16"/>
+      <c r="H93" s="16"/>
+      <c r="I93" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
         <v>292</v>
       </c>
@@ -4471,13 +4916,16 @@
       <c r="E94" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F94" s="14">
+      <c r="F94" s="16">
         <v>12</v>
       </c>
-      <c r="G94" s="14"/>
-      <c r="H94" s="14"/>
-    </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G94" s="16"/>
+      <c r="H94" s="16"/>
+      <c r="I94" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" s="7" t="s">
         <v>295</v>
       </c>
@@ -4493,13 +4941,16 @@
       <c r="E95" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F95" s="14">
+      <c r="F95" s="16">
         <v>12</v>
       </c>
-      <c r="G95" s="14"/>
-      <c r="H95" s="14"/>
-    </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G95" s="16"/>
+      <c r="H95" s="16"/>
+      <c r="I95" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>298</v>
       </c>
@@ -4515,13 +4966,16 @@
       <c r="E96" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F96" s="14">
+      <c r="F96" s="16">
         <v>10</v>
       </c>
-      <c r="G96" s="14"/>
-      <c r="H96" s="14"/>
-    </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G96" s="16"/>
+      <c r="H96" s="16"/>
+      <c r="I96" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" s="7" t="s">
         <v>300</v>
       </c>
@@ -4537,13 +4991,16 @@
       <c r="E97" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F97" s="14">
+      <c r="F97" s="16">
         <v>14</v>
       </c>
-      <c r="G97" s="14"/>
-      <c r="H97" s="14"/>
-    </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G97" s="16"/>
+      <c r="H97" s="16"/>
+      <c r="I97" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
         <v>303</v>
       </c>
@@ -4559,13 +5016,16 @@
       <c r="E98" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F98" s="14">
+      <c r="F98" s="16">
         <v>15</v>
       </c>
-      <c r="G98" s="14"/>
-      <c r="H98" s="14"/>
-    </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G98" s="16"/>
+      <c r="H98" s="16"/>
+      <c r="I98" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" s="7" t="s">
         <v>306</v>
       </c>
@@ -4581,13 +5041,16 @@
       <c r="E99" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F99" s="14">
+      <c r="F99" s="16">
         <v>15</v>
       </c>
-      <c r="G99" s="14"/>
-      <c r="H99" s="14"/>
-    </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G99" s="16"/>
+      <c r="H99" s="16"/>
+      <c r="I99" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
         <v>309</v>
       </c>
@@ -4603,13 +5066,16 @@
       <c r="E100" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F100" s="14">
+      <c r="F100" s="16">
         <v>14</v>
       </c>
-      <c r="G100" s="14"/>
-      <c r="H100" s="14"/>
-    </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G100" s="16"/>
+      <c r="H100" s="16"/>
+      <c r="I100" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" s="7" t="s">
         <v>312</v>
       </c>
@@ -4625,13 +5091,16 @@
       <c r="E101" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F101" s="14">
+      <c r="F101" s="16">
         <v>15</v>
       </c>
-      <c r="G101" s="14"/>
-      <c r="H101" s="14"/>
-    </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G101" s="16"/>
+      <c r="H101" s="16"/>
+      <c r="I101" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
         <v>315</v>
       </c>
@@ -4647,13 +5116,16 @@
       <c r="E102" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F102" s="14">
+      <c r="F102" s="16">
         <v>4</v>
       </c>
-      <c r="G102" s="14"/>
-      <c r="H102" s="14"/>
-    </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G102" s="16"/>
+      <c r="H102" s="16"/>
+      <c r="I102" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" s="7" t="s">
         <v>319</v>
       </c>
@@ -4669,13 +5141,16 @@
       <c r="E103" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F103" s="14">
+      <c r="F103" s="16">
         <v>6</v>
       </c>
-      <c r="G103" s="14"/>
-      <c r="H103" s="14"/>
-    </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G103" s="16"/>
+      <c r="H103" s="16"/>
+      <c r="I103" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>322</v>
       </c>
@@ -4691,13 +5166,16 @@
       <c r="E104" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F104" s="14">
+      <c r="F104" s="16">
         <v>7</v>
       </c>
-      <c r="G104" s="14"/>
-      <c r="H104" s="14"/>
-    </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G104" s="16"/>
+      <c r="H104" s="16"/>
+      <c r="I104" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" s="7" t="s">
         <v>325</v>
       </c>
@@ -4713,17 +5191,20 @@
       <c r="E105" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="F105" s="14">
+      <c r="F105" s="16">
         <v>1</v>
       </c>
-      <c r="G105" s="14">
+      <c r="G105" s="16">
         <v>3</v>
       </c>
-      <c r="H105" s="14">
+      <c r="H105" s="16">
         <v>6</v>
       </c>
-    </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I105" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
         <v>328</v>
       </c>
@@ -4739,13 +5220,16 @@
       <c r="E106" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F106" s="14">
+      <c r="F106" s="16">
         <v>5</v>
       </c>
-      <c r="G106" s="14"/>
-      <c r="H106" s="14"/>
-    </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G106" s="16"/>
+      <c r="H106" s="16"/>
+      <c r="I106" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" s="7" t="s">
         <v>331</v>
       </c>
@@ -4761,13 +5245,16 @@
       <c r="E107" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F107" s="14">
+      <c r="F107" s="16">
         <v>3</v>
       </c>
-      <c r="G107" s="14"/>
-      <c r="H107" s="14"/>
-    </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G107" s="16"/>
+      <c r="H107" s="16"/>
+      <c r="I107" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
         <v>334</v>
       </c>
@@ -4783,13 +5270,16 @@
       <c r="E108" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F108" s="14">
+      <c r="F108" s="16">
         <v>5</v>
       </c>
-      <c r="G108" s="14"/>
-      <c r="H108" s="14"/>
-    </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G108" s="16"/>
+      <c r="H108" s="16"/>
+      <c r="I108" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109" s="7" t="s">
         <v>337</v>
       </c>
@@ -4805,13 +5295,16 @@
       <c r="E109" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F109" s="14">
+      <c r="F109" s="16">
         <v>6</v>
       </c>
-      <c r="G109" s="14"/>
-      <c r="H109" s="14"/>
-    </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G109" s="16"/>
+      <c r="H109" s="16"/>
+      <c r="I109" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>340</v>
       </c>
@@ -4827,13 +5320,16 @@
       <c r="E110" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F110" s="14">
+      <c r="F110" s="16">
         <v>8</v>
       </c>
-      <c r="G110" s="14"/>
-      <c r="H110" s="14"/>
-    </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G110" s="16"/>
+      <c r="H110" s="16"/>
+      <c r="I110" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A111" s="7" t="s">
         <v>343</v>
       </c>
@@ -4849,13 +5345,16 @@
       <c r="E111" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F111" s="14">
+      <c r="F111" s="16">
         <v>4</v>
       </c>
-      <c r="G111" s="14"/>
-      <c r="H111" s="14"/>
-    </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G111" s="16"/>
+      <c r="H111" s="16"/>
+      <c r="I111" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
         <v>346</v>
       </c>
@@ -4871,13 +5370,16 @@
       <c r="E112" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F112" s="14">
+      <c r="F112" s="16">
         <v>5</v>
       </c>
-      <c r="G112" s="14"/>
-      <c r="H112" s="14"/>
-    </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G112" s="16"/>
+      <c r="H112" s="16"/>
+      <c r="I112" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A113" s="7" t="s">
         <v>350</v>
       </c>
@@ -4893,13 +5395,16 @@
       <c r="E113" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F113" s="14">
+      <c r="F113" s="16">
         <v>3</v>
       </c>
-      <c r="G113" s="14"/>
-      <c r="H113" s="14"/>
-    </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G113" s="16"/>
+      <c r="H113" s="16"/>
+      <c r="I113" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
         <v>353</v>
       </c>
@@ -4915,13 +5420,16 @@
       <c r="E114" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F114" s="14">
+      <c r="F114" s="16">
         <v>6</v>
       </c>
-      <c r="G114" s="14"/>
-      <c r="H114" s="14"/>
-    </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G114" s="16"/>
+      <c r="H114" s="16"/>
+      <c r="I114" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A115" s="7" t="s">
         <v>356</v>
       </c>
@@ -4937,13 +5445,16 @@
       <c r="E115" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F115" s="14">
+      <c r="F115" s="16">
         <v>5</v>
       </c>
-      <c r="G115" s="14"/>
-      <c r="H115" s="14"/>
-    </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G115" s="16"/>
+      <c r="H115" s="16"/>
+      <c r="I115" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
         <v>359</v>
       </c>
@@ -4959,13 +5470,16 @@
       <c r="E116" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F116" s="14">
+      <c r="F116" s="16">
         <v>7</v>
       </c>
-      <c r="G116" s="14"/>
-      <c r="H116" s="14"/>
-    </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G116" s="16"/>
+      <c r="H116" s="16"/>
+      <c r="I116" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A117" s="7" t="s">
         <v>362</v>
       </c>
@@ -4981,13 +5495,16 @@
       <c r="E117" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F117" s="14">
+      <c r="F117" s="16">
         <v>4</v>
       </c>
-      <c r="G117" s="14"/>
-      <c r="H117" s="14"/>
-    </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G117" s="16"/>
+      <c r="H117" s="16"/>
+      <c r="I117" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>365</v>
       </c>
@@ -5003,13 +5520,16 @@
       <c r="E118" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F118" s="14">
+      <c r="F118" s="16">
         <v>6</v>
       </c>
-      <c r="G118" s="14"/>
-      <c r="H118" s="14"/>
-    </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G118" s="16"/>
+      <c r="H118" s="16"/>
+      <c r="I118" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A119" s="7" t="s">
         <v>368</v>
       </c>
@@ -5025,13 +5545,16 @@
       <c r="E119" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F119" s="14">
-        <v>9</v>
-      </c>
-      <c r="G119" s="14"/>
-      <c r="H119" s="14"/>
-    </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F119" s="16">
+        <v>9</v>
+      </c>
+      <c r="G119" s="16"/>
+      <c r="H119" s="16"/>
+      <c r="I119" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
         <v>371</v>
       </c>
@@ -5047,13 +5570,16 @@
       <c r="E120" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F120" s="14">
+      <c r="F120" s="16">
         <v>5</v>
       </c>
-      <c r="G120" s="14"/>
-      <c r="H120" s="14"/>
-    </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G120" s="16"/>
+      <c r="H120" s="16"/>
+      <c r="I120" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121" s="7" t="s">
         <v>375</v>
       </c>
@@ -5069,13 +5595,16 @@
       <c r="E121" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F121" s="14">
+      <c r="F121" s="16">
         <v>6</v>
       </c>
-      <c r="G121" s="14"/>
-      <c r="H121" s="14"/>
-    </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G121" s="16"/>
+      <c r="H121" s="16"/>
+      <c r="I121" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
         <v>378</v>
       </c>
@@ -5091,13 +5620,16 @@
       <c r="E122" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F122" s="14">
+      <c r="F122" s="16">
         <v>6</v>
       </c>
-      <c r="G122" s="14"/>
-      <c r="H122" s="14"/>
-    </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G122" s="16"/>
+      <c r="H122" s="16"/>
+      <c r="I122" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A123" s="7" t="s">
         <v>381</v>
       </c>
@@ -5113,13 +5645,16 @@
       <c r="E123" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F123" s="14">
+      <c r="F123" s="16">
         <v>7</v>
       </c>
-      <c r="G123" s="14"/>
-      <c r="H123" s="14"/>
-    </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G123" s="16"/>
+      <c r="H123" s="16"/>
+      <c r="I123" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
         <v>384</v>
       </c>
@@ -5135,13 +5670,16 @@
       <c r="E124" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F124" s="14">
+      <c r="F124" s="16">
         <v>4</v>
       </c>
-      <c r="G124" s="14"/>
-      <c r="H124" s="14"/>
-    </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G124" s="16"/>
+      <c r="H124" s="16"/>
+      <c r="I124" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A125" s="7" t="s">
         <v>387</v>
       </c>
@@ -5157,13 +5695,16 @@
       <c r="E125" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F125" s="14">
+      <c r="F125" s="16">
         <v>5</v>
       </c>
-      <c r="G125" s="14"/>
-      <c r="H125" s="14"/>
-    </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G125" s="16"/>
+      <c r="H125" s="16"/>
+      <c r="I125" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
         <v>390</v>
       </c>
@@ -5179,13 +5720,16 @@
       <c r="E126" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F126" s="14">
+      <c r="F126" s="16">
         <v>8</v>
       </c>
-      <c r="G126" s="14"/>
-      <c r="H126" s="14"/>
-    </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G126" s="16"/>
+      <c r="H126" s="16"/>
+      <c r="I126" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" s="7" t="s">
         <v>393</v>
       </c>
@@ -5201,13 +5745,16 @@
       <c r="E127" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F127" s="14">
-        <v>9</v>
-      </c>
-      <c r="G127" s="14"/>
-      <c r="H127" s="14"/>
-    </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F127" s="16">
+        <v>9</v>
+      </c>
+      <c r="G127" s="16"/>
+      <c r="H127" s="16"/>
+      <c r="I127" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
         <v>396</v>
       </c>
@@ -5223,13 +5770,16 @@
       <c r="E128" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F128" s="14">
+      <c r="F128" s="16">
         <v>5</v>
       </c>
-      <c r="G128" s="14"/>
-      <c r="H128" s="14"/>
-    </row>
-    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G128" s="16"/>
+      <c r="H128" s="16"/>
+      <c r="I128" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A129" s="7" t="s">
         <v>400</v>
       </c>
@@ -5245,13 +5795,16 @@
       <c r="E129" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F129" s="14">
+      <c r="F129" s="16">
         <v>6</v>
       </c>
-      <c r="G129" s="14"/>
-      <c r="H129" s="14"/>
-    </row>
-    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G129" s="16"/>
+      <c r="H129" s="16"/>
+      <c r="I129" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="130" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
         <v>403</v>
       </c>
@@ -5267,13 +5820,16 @@
       <c r="E130" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F130" s="14">
+      <c r="F130" s="16">
         <v>6</v>
       </c>
-      <c r="G130" s="14"/>
-      <c r="H130" s="14"/>
-    </row>
-    <row r="131" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G130" s="16"/>
+      <c r="H130" s="16"/>
+      <c r="I130" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="131" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A131" s="7" t="s">
         <v>406</v>
       </c>
@@ -5289,13 +5845,16 @@
       <c r="E131" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F131" s="14">
+      <c r="F131" s="16">
         <v>4</v>
       </c>
-      <c r="G131" s="14"/>
-      <c r="H131" s="14"/>
-    </row>
-    <row r="132" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G131" s="16"/>
+      <c r="H131" s="16"/>
+      <c r="I131" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="132" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
         <v>409</v>
       </c>
@@ -5311,13 +5870,16 @@
       <c r="E132" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F132" s="14">
+      <c r="F132" s="16">
         <v>7</v>
       </c>
-      <c r="G132" s="14"/>
-      <c r="H132" s="14"/>
-    </row>
-    <row r="133" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G132" s="16"/>
+      <c r="H132" s="16"/>
+      <c r="I132" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="133" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A133" s="7" t="s">
         <v>412</v>
       </c>
@@ -5333,13 +5895,16 @@
       <c r="E133" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F133" s="14">
+      <c r="F133" s="16">
         <v>5</v>
       </c>
-      <c r="G133" s="14"/>
-      <c r="H133" s="14"/>
-    </row>
-    <row r="134" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G133" s="16"/>
+      <c r="H133" s="16"/>
+      <c r="I133" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
         <v>415</v>
       </c>
@@ -5355,17 +5920,20 @@
       <c r="E134" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="F134" s="14">
+      <c r="F134" s="16">
         <v>1</v>
       </c>
-      <c r="G134" s="14">
+      <c r="G134" s="16">
         <v>4</v>
       </c>
-      <c r="H134" s="14">
+      <c r="H134" s="16">
         <v>8</v>
       </c>
-    </row>
-    <row r="135" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I134" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="135" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A135" s="7" t="s">
         <v>418</v>
       </c>
@@ -5381,13 +5949,16 @@
       <c r="E135" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F135" s="14">
-        <v>9</v>
-      </c>
-      <c r="G135" s="14"/>
-      <c r="H135" s="14"/>
-    </row>
-    <row r="136" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F135" s="16">
+        <v>9</v>
+      </c>
+      <c r="G135" s="16"/>
+      <c r="H135" s="16"/>
+      <c r="I135" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
         <v>421</v>
       </c>
@@ -5403,13 +5974,16 @@
       <c r="E136" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F136" s="14">
+      <c r="F136" s="16">
         <v>5</v>
       </c>
-      <c r="G136" s="14"/>
-      <c r="H136" s="14"/>
-    </row>
-    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G136" s="16"/>
+      <c r="H136" s="16"/>
+      <c r="I136" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" s="7" t="s">
         <v>425</v>
       </c>
@@ -5425,13 +5999,16 @@
       <c r="E137" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F137" s="14">
+      <c r="F137" s="16">
         <v>6</v>
       </c>
-      <c r="G137" s="14"/>
-      <c r="H137" s="14"/>
-    </row>
-    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G137" s="16"/>
+      <c r="H137" s="16"/>
+      <c r="I137" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
         <v>428</v>
       </c>
@@ -5447,13 +6024,16 @@
       <c r="E138" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F138" s="14">
+      <c r="F138" s="16">
         <v>7</v>
       </c>
-      <c r="G138" s="14"/>
-      <c r="H138" s="14"/>
-    </row>
-    <row r="139" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G138" s="16"/>
+      <c r="H138" s="16"/>
+      <c r="I138" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="139" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A139" s="7" t="s">
         <v>431</v>
       </c>
@@ -5469,13 +6049,16 @@
       <c r="E139" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F139" s="14">
+      <c r="F139" s="16">
         <v>6</v>
       </c>
-      <c r="G139" s="14"/>
-      <c r="H139" s="14"/>
-    </row>
-    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G139" s="16"/>
+      <c r="H139" s="16"/>
+      <c r="I139" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
         <v>434</v>
       </c>
@@ -5491,13 +6074,16 @@
       <c r="E140" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F140" s="14">
+      <c r="F140" s="16">
         <v>8</v>
       </c>
-      <c r="G140" s="14"/>
-      <c r="H140" s="14"/>
-    </row>
-    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G140" s="16"/>
+      <c r="H140" s="16"/>
+      <c r="I140" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" s="7" t="s">
         <v>437</v>
       </c>
@@ -5513,13 +6099,16 @@
       <c r="E141" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F141" s="14">
+      <c r="F141" s="16">
         <v>7</v>
       </c>
-      <c r="G141" s="14"/>
-      <c r="H141" s="14"/>
-    </row>
-    <row r="142" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G141" s="16"/>
+      <c r="H141" s="16"/>
+      <c r="I141" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
         <v>440</v>
       </c>
@@ -5535,13 +6124,16 @@
       <c r="E142" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F142" s="14">
+      <c r="F142" s="16">
         <v>4</v>
       </c>
-      <c r="G142" s="14"/>
-      <c r="H142" s="14"/>
-    </row>
-    <row r="143" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G142" s="16"/>
+      <c r="H142" s="16"/>
+      <c r="I142" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A143" s="7" t="s">
         <v>443</v>
       </c>
@@ -5557,13 +6149,16 @@
       <c r="E143" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F143" s="14">
-        <v>9</v>
-      </c>
-      <c r="G143" s="14"/>
-      <c r="H143" s="14"/>
-    </row>
-    <row r="144" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F143" s="16">
+        <v>9</v>
+      </c>
+      <c r="G143" s="16"/>
+      <c r="H143" s="16"/>
+      <c r="I143" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
         <v>446</v>
       </c>
@@ -5579,13 +6174,16 @@
       <c r="E144" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F144" s="14">
+      <c r="F144" s="16">
         <v>12</v>
       </c>
-      <c r="G144" s="14"/>
-      <c r="H144" s="14"/>
-    </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G144" s="16"/>
+      <c r="H144" s="16"/>
+      <c r="I144" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A145" s="7" t="s">
         <v>449</v>
       </c>
@@ -5601,13 +6199,16 @@
       <c r="E145" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F145" s="14">
+      <c r="F145" s="16">
         <v>14</v>
       </c>
-      <c r="G145" s="14"/>
-      <c r="H145" s="14"/>
-    </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G145" s="16"/>
+      <c r="H145" s="16"/>
+      <c r="I145" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="146" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
         <v>452</v>
       </c>
@@ -5623,13 +6224,16 @@
       <c r="E146" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F146" s="14">
+      <c r="F146" s="16">
         <v>12</v>
       </c>
-      <c r="G146" s="14"/>
-      <c r="H146" s="14"/>
-    </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G146" s="16"/>
+      <c r="H146" s="16"/>
+      <c r="I146" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A147" s="7" t="s">
         <v>455</v>
       </c>
@@ -5645,13 +6249,16 @@
       <c r="E147" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F147" s="14">
+      <c r="F147" s="16">
         <v>14</v>
       </c>
-      <c r="G147" s="14"/>
-      <c r="H147" s="14"/>
-    </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G147" s="16"/>
+      <c r="H147" s="16"/>
+      <c r="I147" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
         <v>458</v>
       </c>
@@ -5667,13 +6274,16 @@
       <c r="E148" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F148" s="14">
+      <c r="F148" s="16">
         <v>12</v>
       </c>
-      <c r="G148" s="14"/>
-      <c r="H148" s="14"/>
-    </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G148" s="16"/>
+      <c r="H148" s="16"/>
+      <c r="I148" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A149" s="7" t="s">
         <v>461</v>
       </c>
@@ -5689,13 +6299,16 @@
       <c r="E149" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F149" s="14">
+      <c r="F149" s="16">
         <v>13</v>
       </c>
-      <c r="G149" s="14"/>
-      <c r="H149" s="14"/>
-    </row>
-    <row r="150" spans="1:8" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="G149" s="16"/>
+      <c r="H149" s="16"/>
+      <c r="I149" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="150" spans="1:9" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
         <v>464</v>
       </c>
@@ -5711,13 +6324,16 @@
       <c r="E150" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F150" s="14">
+      <c r="F150" s="16">
         <v>15</v>
       </c>
-      <c r="G150" s="14"/>
-      <c r="H150" s="14"/>
-    </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G150" s="16"/>
+      <c r="H150" s="16"/>
+      <c r="I150" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A151" s="7" t="s">
         <v>467</v>
       </c>
@@ -5733,13 +6349,16 @@
       <c r="E151" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F151" s="14">
+      <c r="F151" s="16">
         <v>15</v>
       </c>
-      <c r="G151" s="14"/>
-      <c r="H151" s="14"/>
-    </row>
-    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G151" s="16"/>
+      <c r="H151" s="16"/>
+      <c r="I151" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="152" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
         <v>470</v>
       </c>
@@ -5755,13 +6374,16 @@
       <c r="E152" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F152" s="14">
+      <c r="F152" s="16">
         <v>6</v>
       </c>
-      <c r="G152" s="14"/>
-      <c r="H152" s="14"/>
-    </row>
-    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G152" s="16"/>
+      <c r="H152" s="16"/>
+      <c r="I152" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="153" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A153" s="7" t="s">
         <v>474</v>
       </c>
@@ -5777,17 +6399,20 @@
       <c r="E153" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="F153" s="14">
+      <c r="F153" s="16">
         <v>1</v>
       </c>
-      <c r="G153" s="14">
+      <c r="G153" s="16">
         <v>2</v>
       </c>
-      <c r="H153" s="14">
+      <c r="H153" s="16">
         <v>4</v>
       </c>
-    </row>
-    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I153" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
         <v>477</v>
       </c>
@@ -5803,13 +6428,16 @@
       <c r="E154" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F154" s="14">
+      <c r="F154" s="16">
         <v>6</v>
       </c>
-      <c r="G154" s="14"/>
-      <c r="H154" s="14"/>
-    </row>
-    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G154" s="16"/>
+      <c r="H154" s="16"/>
+      <c r="I154" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="155" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A155" s="7" t="s">
         <v>480</v>
       </c>
@@ -5825,17 +6453,20 @@
       <c r="E155" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="F155" s="14">
+      <c r="F155" s="16">
         <v>1</v>
       </c>
-      <c r="G155" s="14">
+      <c r="G155" s="16">
         <v>3</v>
       </c>
-      <c r="H155" s="14">
+      <c r="H155" s="16">
         <v>7</v>
       </c>
-    </row>
-    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I155" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="156" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
         <v>483</v>
       </c>
@@ -5851,13 +6482,16 @@
       <c r="E156" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F156" s="14">
+      <c r="F156" s="16">
         <v>8</v>
       </c>
-      <c r="G156" s="14"/>
-      <c r="H156" s="14"/>
-    </row>
-    <row r="157" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G156" s="16"/>
+      <c r="H156" s="16"/>
+      <c r="I156" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="157" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A157" s="7" t="s">
         <v>486</v>
       </c>
@@ -5873,17 +6507,20 @@
       <c r="E157" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="F157" s="14">
+      <c r="F157" s="16">
         <v>1</v>
       </c>
-      <c r="G157" s="14">
+      <c r="G157" s="16">
         <v>4</v>
       </c>
-      <c r="H157" s="14">
+      <c r="H157" s="16">
         <v>8</v>
       </c>
-    </row>
-    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I157" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="158" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
         <v>489</v>
       </c>
@@ -5899,13 +6536,16 @@
       <c r="E158" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F158" s="14">
+      <c r="F158" s="16">
         <v>6</v>
       </c>
-      <c r="G158" s="14"/>
-      <c r="H158" s="14"/>
-    </row>
-    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G158" s="16"/>
+      <c r="H158" s="16"/>
+      <c r="I158" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="159" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A159" s="7" t="s">
         <v>492</v>
       </c>
@@ -5921,17 +6561,20 @@
       <c r="E159" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="F159" s="14">
+      <c r="F159" s="16">
         <v>1</v>
       </c>
-      <c r="G159" s="14">
+      <c r="G159" s="16">
         <v>4</v>
       </c>
-      <c r="H159" s="14">
+      <c r="H159" s="16">
         <v>8</v>
       </c>
-    </row>
-    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I159" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="160" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
         <v>495</v>
       </c>
@@ -5947,13 +6590,16 @@
       <c r="E160" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F160" s="14">
-        <v>9</v>
-      </c>
-      <c r="G160" s="14"/>
-      <c r="H160" s="14"/>
-    </row>
-    <row r="161" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F160" s="16">
+        <v>9</v>
+      </c>
+      <c r="G160" s="16"/>
+      <c r="H160" s="16"/>
+      <c r="I160" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="161" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A161" s="7" t="s">
         <v>498</v>
       </c>
@@ -5969,13 +6615,16 @@
       <c r="E161" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F161" s="14">
+      <c r="F161" s="16">
         <v>4</v>
       </c>
-      <c r="G161" s="14"/>
-      <c r="H161" s="14"/>
-    </row>
-    <row r="162" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G161" s="16"/>
+      <c r="H161" s="16"/>
+      <c r="I161" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="162" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
         <v>501</v>
       </c>
@@ -5991,13 +6640,16 @@
       <c r="E162" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F162" s="14">
+      <c r="F162" s="16">
         <v>5</v>
       </c>
-      <c r="G162" s="14"/>
-      <c r="H162" s="14"/>
-    </row>
-    <row r="163" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G162" s="16"/>
+      <c r="H162" s="16"/>
+      <c r="I162" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="163" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A163" s="7" t="s">
         <v>505</v>
       </c>
@@ -6013,13 +6665,16 @@
       <c r="E163" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F163" s="14">
+      <c r="F163" s="16">
         <v>6</v>
       </c>
-      <c r="G163" s="14"/>
-      <c r="H163" s="14"/>
-    </row>
-    <row r="164" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G163" s="16"/>
+      <c r="H163" s="16"/>
+      <c r="I163" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="164" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
         <v>508</v>
       </c>
@@ -6035,13 +6690,16 @@
       <c r="E164" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F164" s="14">
+      <c r="F164" s="16">
         <v>4</v>
       </c>
-      <c r="G164" s="14"/>
-      <c r="H164" s="14"/>
-    </row>
-    <row r="165" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G164" s="16"/>
+      <c r="H164" s="16"/>
+      <c r="I164" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="165" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A165" s="7" t="s">
         <v>510</v>
       </c>
@@ -6057,13 +6715,16 @@
       <c r="E165" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F165" s="14">
+      <c r="F165" s="16">
         <v>6</v>
       </c>
-      <c r="G165" s="14"/>
-      <c r="H165" s="14"/>
-    </row>
-    <row r="166" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G165" s="16"/>
+      <c r="H165" s="16"/>
+      <c r="I165" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="166" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
         <v>513</v>
       </c>
@@ -6079,13 +6740,16 @@
       <c r="E166" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F166" s="14">
+      <c r="F166" s="16">
         <v>8</v>
       </c>
-      <c r="G166" s="14"/>
-      <c r="H166" s="14"/>
-    </row>
-    <row r="167" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G166" s="16"/>
+      <c r="H166" s="16"/>
+      <c r="I166" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="167" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A167" s="7" t="s">
         <v>516</v>
       </c>
@@ -6101,13 +6765,16 @@
       <c r="E167" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F167" s="14">
+      <c r="F167" s="16">
         <v>3</v>
       </c>
-      <c r="G167" s="14"/>
-      <c r="H167" s="14"/>
-    </row>
-    <row r="168" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G167" s="16"/>
+      <c r="H167" s="16"/>
+      <c r="I167" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="168" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
         <v>519</v>
       </c>
@@ -6123,13 +6790,16 @@
       <c r="E168" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F168" s="14">
+      <c r="F168" s="16">
         <v>7</v>
       </c>
-      <c r="G168" s="14"/>
-      <c r="H168" s="14"/>
-    </row>
-    <row r="169" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G168" s="16"/>
+      <c r="H168" s="16"/>
+      <c r="I168" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="169" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A169" s="7" t="s">
         <v>522</v>
       </c>
@@ -6145,13 +6815,16 @@
       <c r="E169" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F169" s="14">
-        <v>9</v>
-      </c>
-      <c r="G169" s="14"/>
-      <c r="H169" s="14"/>
-    </row>
-    <row r="170" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F169" s="16">
+        <v>9</v>
+      </c>
+      <c r="G169" s="16"/>
+      <c r="H169" s="16"/>
+      <c r="I169" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="170" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
         <v>525</v>
       </c>
@@ -6167,13 +6840,16 @@
       <c r="E170" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F170" s="14">
+      <c r="F170" s="16">
         <v>5</v>
       </c>
-      <c r="G170" s="14"/>
-      <c r="H170" s="14"/>
-    </row>
-    <row r="171" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G170" s="16"/>
+      <c r="H170" s="16"/>
+      <c r="I170" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="171" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A171" s="7" t="s">
         <v>529</v>
       </c>
@@ -6189,13 +6865,16 @@
       <c r="E171" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F171" s="14">
+      <c r="F171" s="16">
         <v>6</v>
       </c>
-      <c r="G171" s="14"/>
-      <c r="H171" s="14"/>
-    </row>
-    <row r="172" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G171" s="16"/>
+      <c r="H171" s="16"/>
+      <c r="I171" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="172" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
         <v>532</v>
       </c>
@@ -6211,13 +6890,16 @@
       <c r="E172" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F172" s="14">
+      <c r="F172" s="16">
         <v>4</v>
       </c>
-      <c r="G172" s="14"/>
-      <c r="H172" s="14"/>
-    </row>
-    <row r="173" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G172" s="16"/>
+      <c r="H172" s="16"/>
+      <c r="I172" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="173" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A173" s="7" t="s">
         <v>535</v>
       </c>
@@ -6233,13 +6915,16 @@
       <c r="E173" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F173" s="14">
+      <c r="F173" s="16">
         <v>6</v>
       </c>
-      <c r="G173" s="14"/>
-      <c r="H173" s="14"/>
-    </row>
-    <row r="174" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G173" s="16"/>
+      <c r="H173" s="16"/>
+      <c r="I173" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="174" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
         <v>538</v>
       </c>
@@ -6255,13 +6940,16 @@
       <c r="E174" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F174" s="14">
+      <c r="F174" s="16">
         <v>8</v>
       </c>
-      <c r="G174" s="14"/>
-      <c r="H174" s="14"/>
-    </row>
-    <row r="175" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G174" s="16"/>
+      <c r="H174" s="16"/>
+      <c r="I174" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="175" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A175" s="7" t="s">
         <v>541</v>
       </c>
@@ -6277,13 +6965,16 @@
       <c r="E175" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F175" s="14">
+      <c r="F175" s="16">
         <v>5</v>
       </c>
-      <c r="G175" s="14"/>
-      <c r="H175" s="14"/>
-    </row>
-    <row r="176" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G175" s="16"/>
+      <c r="H175" s="16"/>
+      <c r="I175" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="176" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
         <v>544</v>
       </c>
@@ -6299,13 +6990,16 @@
       <c r="E176" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F176" s="14">
+      <c r="F176" s="16">
         <v>7</v>
       </c>
-      <c r="G176" s="14"/>
-      <c r="H176" s="14"/>
-    </row>
-    <row r="177" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G176" s="16"/>
+      <c r="H176" s="16"/>
+      <c r="I176" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="177" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A177" s="7" t="s">
         <v>547</v>
       </c>
@@ -6321,13 +7015,16 @@
       <c r="E177" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F177" s="14">
-        <v>9</v>
-      </c>
-      <c r="G177" s="14"/>
-      <c r="H177" s="14"/>
-    </row>
-    <row r="178" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F177" s="16">
+        <v>9</v>
+      </c>
+      <c r="G177" s="16"/>
+      <c r="H177" s="16"/>
+      <c r="I177" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="178" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
         <v>550</v>
       </c>
@@ -6343,13 +7040,16 @@
       <c r="E178" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F178" s="14">
+      <c r="F178" s="16">
         <v>5</v>
       </c>
-      <c r="G178" s="14"/>
-      <c r="H178" s="14"/>
-    </row>
-    <row r="179" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G178" s="16"/>
+      <c r="H178" s="16"/>
+      <c r="I178" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="179" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A179" s="7" t="s">
         <v>554</v>
       </c>
@@ -6365,17 +7065,20 @@
       <c r="E179" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="F179" s="14">
+      <c r="F179" s="16">
         <v>1</v>
       </c>
-      <c r="G179" s="14">
+      <c r="G179" s="16">
         <v>3</v>
       </c>
-      <c r="H179" s="14">
+      <c r="H179" s="16">
         <v>7</v>
       </c>
-    </row>
-    <row r="180" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I179" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="180" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
         <v>557</v>
       </c>
@@ -6391,13 +7094,16 @@
       <c r="E180" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F180" s="14">
+      <c r="F180" s="16">
         <v>4</v>
       </c>
-      <c r="G180" s="14"/>
-      <c r="H180" s="14"/>
-    </row>
-    <row r="181" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G180" s="16"/>
+      <c r="H180" s="16"/>
+      <c r="I180" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="181" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A181" s="7" t="s">
         <v>560</v>
       </c>
@@ -6413,17 +7119,20 @@
       <c r="E181" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="F181" s="14">
+      <c r="F181" s="16">
         <v>1</v>
       </c>
-      <c r="G181" s="14">
+      <c r="G181" s="16">
         <v>4</v>
       </c>
-      <c r="H181" s="14">
+      <c r="H181" s="16">
         <v>8</v>
       </c>
-    </row>
-    <row r="182" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I181" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="182" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
         <v>563</v>
       </c>
@@ -6439,13 +7148,16 @@
       <c r="E182" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F182" s="14">
+      <c r="F182" s="16">
         <v>6</v>
       </c>
-      <c r="G182" s="14"/>
-      <c r="H182" s="14"/>
-    </row>
-    <row r="183" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G182" s="16"/>
+      <c r="H182" s="16"/>
+      <c r="I182" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="183" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A183" s="7" t="s">
         <v>566</v>
       </c>
@@ -6461,13 +7173,16 @@
       <c r="E183" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F183" s="14">
+      <c r="F183" s="16">
         <v>5</v>
       </c>
-      <c r="G183" s="14"/>
-      <c r="H183" s="14"/>
-    </row>
-    <row r="184" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G183" s="16"/>
+      <c r="H183" s="16"/>
+      <c r="I183" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="184" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
         <v>568</v>
       </c>
@@ -6483,13 +7198,16 @@
       <c r="E184" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F184" s="14">
+      <c r="F184" s="16">
         <v>7</v>
       </c>
-      <c r="G184" s="14"/>
-      <c r="H184" s="14"/>
-    </row>
-    <row r="185" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G184" s="16"/>
+      <c r="H184" s="16"/>
+      <c r="I184" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="185" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A185" s="7" t="s">
         <v>571</v>
       </c>
@@ -6505,13 +7223,16 @@
       <c r="E185" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F185" s="14">
-        <v>9</v>
-      </c>
-      <c r="G185" s="14"/>
-      <c r="H185" s="14"/>
-    </row>
-    <row r="186" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F185" s="16">
+        <v>9</v>
+      </c>
+      <c r="G185" s="16"/>
+      <c r="H185" s="16"/>
+      <c r="I185" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="186" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
         <v>574</v>
       </c>
@@ -6527,13 +7248,16 @@
       <c r="E186" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F186" s="14">
+      <c r="F186" s="16">
         <v>5</v>
       </c>
-      <c r="G186" s="14"/>
-      <c r="H186" s="14"/>
-    </row>
-    <row r="187" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G186" s="16"/>
+      <c r="H186" s="16"/>
+      <c r="I186" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="187" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A187" s="7" t="s">
         <v>578</v>
       </c>
@@ -6549,13 +7273,16 @@
       <c r="E187" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F187" s="14">
+      <c r="F187" s="16">
         <v>6</v>
       </c>
-      <c r="G187" s="14"/>
-      <c r="H187" s="14"/>
-    </row>
-    <row r="188" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G187" s="16"/>
+      <c r="H187" s="16"/>
+      <c r="I187" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="188" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
         <v>581</v>
       </c>
@@ -6571,17 +7298,20 @@
       <c r="E188" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="F188" s="14">
+      <c r="F188" s="16">
         <v>2</v>
       </c>
-      <c r="G188" s="14">
+      <c r="G188" s="16">
         <v>5</v>
       </c>
-      <c r="H188" s="14">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="189" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H188" s="16">
+        <v>9</v>
+      </c>
+      <c r="I188" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="189" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A189" s="7" t="s">
         <v>584</v>
       </c>
@@ -6597,13 +7327,16 @@
       <c r="E189" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F189" s="14">
+      <c r="F189" s="16">
         <v>6</v>
       </c>
-      <c r="G189" s="14"/>
-      <c r="H189" s="14"/>
-    </row>
-    <row r="190" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G189" s="16"/>
+      <c r="H189" s="16"/>
+      <c r="I189" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="190" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
         <v>587</v>
       </c>
@@ -6619,13 +7352,16 @@
       <c r="E190" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F190" s="14">
+      <c r="F190" s="16">
         <v>8</v>
       </c>
-      <c r="G190" s="14"/>
-      <c r="H190" s="14"/>
-    </row>
-    <row r="191" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G190" s="16"/>
+      <c r="H190" s="16"/>
+      <c r="I190" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="191" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A191" s="7" t="s">
         <v>590</v>
       </c>
@@ -6641,13 +7377,16 @@
       <c r="E191" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F191" s="14">
+      <c r="F191" s="16">
         <v>4</v>
       </c>
-      <c r="G191" s="14"/>
-      <c r="H191" s="14"/>
-    </row>
-    <row r="192" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G191" s="16"/>
+      <c r="H191" s="16"/>
+      <c r="I191" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="192" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
         <v>593</v>
       </c>
@@ -6663,13 +7402,16 @@
       <c r="E192" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F192" s="14">
+      <c r="F192" s="16">
         <v>7</v>
       </c>
-      <c r="G192" s="14"/>
-      <c r="H192" s="14"/>
-    </row>
-    <row r="193" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G192" s="16"/>
+      <c r="H192" s="16"/>
+      <c r="I192" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="193" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A193" s="7" t="s">
         <v>596</v>
       </c>
@@ -6685,13 +7427,16 @@
       <c r="E193" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F193" s="14">
-        <v>9</v>
-      </c>
-      <c r="G193" s="14"/>
-      <c r="H193" s="14"/>
-    </row>
-    <row r="194" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F193" s="16">
+        <v>9</v>
+      </c>
+      <c r="G193" s="16"/>
+      <c r="H193" s="16"/>
+      <c r="I193" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="194" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
         <v>599</v>
       </c>
@@ -6707,13 +7452,16 @@
       <c r="E194" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F194" s="14">
+      <c r="F194" s="16">
         <v>12</v>
       </c>
-      <c r="G194" s="14"/>
-      <c r="H194" s="14"/>
-    </row>
-    <row r="195" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G194" s="16"/>
+      <c r="H194" s="16"/>
+      <c r="I194" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="195" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A195" s="7" t="s">
         <v>602</v>
       </c>
@@ -6729,13 +7477,16 @@
       <c r="E195" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F195" s="14">
+      <c r="F195" s="16">
         <v>12</v>
       </c>
-      <c r="G195" s="14"/>
-      <c r="H195" s="14"/>
-    </row>
-    <row r="196" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G195" s="16"/>
+      <c r="H195" s="16"/>
+      <c r="I195" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="196" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
         <v>605</v>
       </c>
@@ -6751,13 +7502,16 @@
       <c r="E196" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F196" s="14">
+      <c r="F196" s="16">
         <v>13</v>
       </c>
-      <c r="G196" s="14"/>
-      <c r="H196" s="14"/>
-    </row>
-    <row r="197" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G196" s="16"/>
+      <c r="H196" s="16"/>
+      <c r="I196" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="197" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A197" s="7" t="s">
         <v>608</v>
       </c>
@@ -6773,13 +7527,16 @@
       <c r="E197" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F197" s="14">
+      <c r="F197" s="16">
         <v>14</v>
       </c>
-      <c r="G197" s="14"/>
-      <c r="H197" s="14"/>
-    </row>
-    <row r="198" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G197" s="16"/>
+      <c r="H197" s="16"/>
+      <c r="I197" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="198" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
         <v>611</v>
       </c>
@@ -6795,13 +7552,16 @@
       <c r="E198" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F198" s="14">
+      <c r="F198" s="16">
         <v>15</v>
       </c>
-      <c r="G198" s="14"/>
-      <c r="H198" s="14"/>
-    </row>
-    <row r="199" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G198" s="16"/>
+      <c r="H198" s="16"/>
+      <c r="I198" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="199" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A199" s="7" t="s">
         <v>614</v>
       </c>
@@ -6817,13 +7577,16 @@
       <c r="E199" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F199" s="14">
+      <c r="F199" s="16">
         <v>15</v>
       </c>
-      <c r="G199" s="14"/>
-      <c r="H199" s="14"/>
-    </row>
-    <row r="200" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G199" s="16"/>
+      <c r="H199" s="16"/>
+      <c r="I199" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="200" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A200" s="2" t="s">
         <v>617</v>
       </c>
@@ -6839,13 +7602,16 @@
       <c r="E200" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F200" s="14">
+      <c r="F200" s="16">
         <v>14</v>
       </c>
-      <c r="G200" s="14"/>
-      <c r="H200" s="14"/>
-    </row>
-    <row r="201" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G200" s="16"/>
+      <c r="H200" s="16"/>
+      <c r="I200" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="201" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A201" s="7" t="s">
         <v>620</v>
       </c>
@@ -6861,13 +7627,16 @@
       <c r="E201" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F201" s="14">
+      <c r="F201" s="16">
         <v>13</v>
       </c>
-      <c r="G201" s="14"/>
-      <c r="H201" s="14"/>
-    </row>
-    <row r="202" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G201" s="16"/>
+      <c r="H201" s="16"/>
+      <c r="I201" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="202" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A202" s="2" t="s">
         <v>623</v>
       </c>
@@ -6883,13 +7652,16 @@
       <c r="E202" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F202" s="14">
+      <c r="F202" s="16">
         <v>3</v>
       </c>
-      <c r="G202" s="14"/>
-      <c r="H202" s="14"/>
-    </row>
-    <row r="203" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G202" s="16"/>
+      <c r="H202" s="16"/>
+      <c r="I202" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="203" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A203" s="7" t="s">
         <v>627</v>
       </c>
@@ -6905,13 +7677,16 @@
       <c r="E203" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F203" s="14">
+      <c r="F203" s="16">
         <v>4</v>
       </c>
-      <c r="G203" s="14"/>
-      <c r="H203" s="14"/>
-    </row>
-    <row r="204" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G203" s="16"/>
+      <c r="H203" s="16"/>
+      <c r="I203" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="204" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A204" s="2" t="s">
         <v>630</v>
       </c>
@@ -6927,13 +7702,16 @@
       <c r="E204" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F204" s="14">
+      <c r="F204" s="16">
         <v>5</v>
       </c>
-      <c r="G204" s="14"/>
-      <c r="H204" s="14"/>
-    </row>
-    <row r="205" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G204" s="16"/>
+      <c r="H204" s="16"/>
+      <c r="I204" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="205" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A205" s="7" t="s">
         <v>633</v>
       </c>
@@ -6949,13 +7727,16 @@
       <c r="E205" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F205" s="14">
-        <v>9</v>
-      </c>
-      <c r="G205" s="14"/>
-      <c r="H205" s="14"/>
-    </row>
-    <row r="206" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F205" s="16">
+        <v>9</v>
+      </c>
+      <c r="G205" s="16"/>
+      <c r="H205" s="16"/>
+      <c r="I205" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="206" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
         <v>636</v>
       </c>
@@ -6971,17 +7752,20 @@
       <c r="E206" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="F206" s="14">
+      <c r="F206" s="16">
         <v>1</v>
       </c>
-      <c r="G206" s="14">
+      <c r="G206" s="16">
         <v>3</v>
       </c>
-      <c r="H206" s="14">
+      <c r="H206" s="16">
         <v>6</v>
       </c>
-    </row>
-    <row r="207" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I206" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="207" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A207" s="7" t="s">
         <v>639</v>
       </c>
@@ -6997,17 +7781,20 @@
       <c r="E207" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="F207" s="14">
+      <c r="F207" s="16">
         <v>1</v>
       </c>
-      <c r="G207" s="14">
+      <c r="G207" s="16">
         <v>3</v>
       </c>
-      <c r="H207" s="14">
+      <c r="H207" s="16">
         <v>6</v>
       </c>
-    </row>
-    <row r="208" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I207" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="208" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
         <v>642</v>
       </c>
@@ -7023,17 +7810,20 @@
       <c r="E208" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="F208" s="14">
+      <c r="F208" s="16">
         <v>1</v>
       </c>
-      <c r="G208" s="14">
+      <c r="G208" s="16">
         <v>3</v>
       </c>
-      <c r="H208" s="14">
+      <c r="H208" s="16">
         <v>6</v>
       </c>
-    </row>
-    <row r="209" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I208" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="209" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A209" s="7" t="s">
         <v>645</v>
       </c>
@@ -7049,17 +7839,20 @@
       <c r="E209" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="F209" s="14">
+      <c r="F209" s="16">
         <v>1</v>
       </c>
-      <c r="G209" s="14">
+      <c r="G209" s="16">
         <v>2</v>
       </c>
-      <c r="H209" s="14">
+      <c r="H209" s="16">
         <v>4</v>
       </c>
-    </row>
-    <row r="210" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I209" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="210" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
         <v>648</v>
       </c>
@@ -7075,17 +7868,20 @@
       <c r="E210" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="F210" s="14">
+      <c r="F210" s="16">
         <v>1</v>
       </c>
-      <c r="G210" s="14">
+      <c r="G210" s="16">
         <v>2</v>
       </c>
-      <c r="H210" s="14">
+      <c r="H210" s="16">
         <v>4</v>
       </c>
-    </row>
-    <row r="211" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I210" s="15" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="211" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A211" s="7" t="s">
         <v>651</v>
       </c>
@@ -7101,14 +7897,17 @@
       <c r="E211" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="F211" s="14">
+      <c r="F211" s="16">
         <v>1</v>
       </c>
-      <c r="G211" s="14">
+      <c r="G211" s="16">
         <v>2</v>
       </c>
-      <c r="H211" s="14">
+      <c r="H211" s="16">
         <v>4</v>
+      </c>
+      <c r="I211" s="15" t="s">
+        <v>659</v>
       </c>
     </row>
   </sheetData>

</xml_diff>